<commit_message>
sql indexing, loading timer, srp compliance tracker May28-June06
</commit_message>
<xml_diff>
--- a/uploads/reports/Zamobanga_City_Full_Report_2025.xlsx
+++ b/uploads/reports/Zamobanga_City_Full_Report_2025.xlsx
@@ -5048,7 +5048,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:G501"/>
+  <dimension ref="A1:G500"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -14015,10 +14015,10 @@
         <v>789</v>
       </c>
       <c r="F390" t="s">
-        <v>239</v>
+        <v>775</v>
       </c>
       <c r="G390" t="s">
-        <v>45</v>
+        <v>790</v>
       </c>
     </row>
     <row r="391" spans="1:7">
@@ -14032,16 +14032,16 @@
         <v>746</v>
       </c>
       <c r="D391" t="s">
-        <v>788</v>
+        <v>791</v>
       </c>
       <c r="E391" t="s">
-        <v>789</v>
+        <v>792</v>
       </c>
       <c r="F391" t="s">
-        <v>775</v>
+        <v>793</v>
       </c>
       <c r="G391" t="s">
-        <v>790</v>
+        <v>45</v>
       </c>
     </row>
     <row r="392" spans="1:7">
@@ -14058,13 +14058,13 @@
         <v>791</v>
       </c>
       <c r="E392" t="s">
-        <v>792</v>
+        <v>794</v>
       </c>
       <c r="F392" t="s">
-        <v>793</v>
+        <v>795</v>
       </c>
       <c r="G392" t="s">
-        <v>45</v>
+        <v>796</v>
       </c>
     </row>
     <row r="393" spans="1:7">
@@ -14084,10 +14084,10 @@
         <v>794</v>
       </c>
       <c r="F393" t="s">
-        <v>795</v>
+        <v>130</v>
       </c>
       <c r="G393" t="s">
-        <v>796</v>
+        <v>797</v>
       </c>
     </row>
     <row r="394" spans="1:7">
@@ -14107,10 +14107,10 @@
         <v>794</v>
       </c>
       <c r="F394" t="s">
-        <v>130</v>
+        <v>798</v>
       </c>
       <c r="G394" t="s">
-        <v>797</v>
+        <v>799</v>
       </c>
     </row>
     <row r="395" spans="1:7">
@@ -14124,16 +14124,16 @@
         <v>746</v>
       </c>
       <c r="D395" t="s">
-        <v>791</v>
+        <v>800</v>
       </c>
       <c r="E395" t="s">
-        <v>794</v>
+        <v>801</v>
       </c>
       <c r="F395" t="s">
-        <v>798</v>
+        <v>627</v>
       </c>
       <c r="G395" t="s">
-        <v>799</v>
+        <v>802</v>
       </c>
     </row>
     <row r="396" spans="1:7">
@@ -14147,16 +14147,16 @@
         <v>746</v>
       </c>
       <c r="D396" t="s">
-        <v>800</v>
+        <v>803</v>
       </c>
       <c r="E396" t="s">
-        <v>801</v>
+        <v>804</v>
       </c>
       <c r="F396" t="s">
-        <v>627</v>
+        <v>239</v>
       </c>
       <c r="G396" t="s">
-        <v>802</v>
+        <v>45</v>
       </c>
     </row>
     <row r="397" spans="1:7">
@@ -14170,10 +14170,10 @@
         <v>746</v>
       </c>
       <c r="D397" t="s">
-        <v>803</v>
+        <v>805</v>
       </c>
       <c r="E397" t="s">
-        <v>804</v>
+        <v>806</v>
       </c>
       <c r="F397" t="s">
         <v>239</v>
@@ -14190,16 +14190,16 @@
         <v>7</v>
       </c>
       <c r="C398" t="s">
-        <v>746</v>
+        <v>807</v>
       </c>
       <c r="D398" t="s">
-        <v>805</v>
+        <v>747</v>
       </c>
       <c r="E398" t="s">
-        <v>806</v>
+        <v>808</v>
       </c>
       <c r="F398" t="s">
-        <v>239</v>
+        <v>809</v>
       </c>
       <c r="G398" t="s">
         <v>45</v>
@@ -14222,10 +14222,10 @@
         <v>808</v>
       </c>
       <c r="F399" t="s">
-        <v>809</v>
+        <v>810</v>
       </c>
       <c r="G399" t="s">
-        <v>45</v>
+        <v>811</v>
       </c>
     </row>
     <row r="400" spans="1:7">
@@ -14245,10 +14245,10 @@
         <v>808</v>
       </c>
       <c r="F400" t="s">
-        <v>810</v>
+        <v>812</v>
       </c>
       <c r="G400" t="s">
-        <v>811</v>
+        <v>813</v>
       </c>
     </row>
     <row r="401" spans="1:7">
@@ -14262,16 +14262,16 @@
         <v>807</v>
       </c>
       <c r="D401" t="s">
-        <v>747</v>
+        <v>757</v>
       </c>
       <c r="E401" t="s">
-        <v>808</v>
+        <v>814</v>
       </c>
       <c r="F401" t="s">
-        <v>812</v>
+        <v>627</v>
       </c>
       <c r="G401" t="s">
-        <v>813</v>
+        <v>815</v>
       </c>
     </row>
     <row r="402" spans="1:7">
@@ -14285,16 +14285,16 @@
         <v>807</v>
       </c>
       <c r="D402" t="s">
-        <v>757</v>
+        <v>816</v>
       </c>
       <c r="E402" t="s">
-        <v>814</v>
+        <v>817</v>
       </c>
       <c r="F402" t="s">
-        <v>627</v>
+        <v>239</v>
       </c>
       <c r="G402" t="s">
-        <v>815</v>
+        <v>818</v>
       </c>
     </row>
     <row r="403" spans="1:7">
@@ -14308,16 +14308,16 @@
         <v>807</v>
       </c>
       <c r="D403" t="s">
-        <v>816</v>
+        <v>819</v>
       </c>
       <c r="E403" t="s">
-        <v>817</v>
+        <v>820</v>
       </c>
       <c r="F403" t="s">
-        <v>239</v>
+        <v>614</v>
       </c>
       <c r="G403" t="s">
-        <v>818</v>
+        <v>821</v>
       </c>
     </row>
     <row r="404" spans="1:7">
@@ -14337,10 +14337,10 @@
         <v>820</v>
       </c>
       <c r="F404" t="s">
-        <v>614</v>
+        <v>798</v>
       </c>
       <c r="G404" t="s">
-        <v>821</v>
+        <v>822</v>
       </c>
     </row>
     <row r="405" spans="1:7">
@@ -14354,16 +14354,16 @@
         <v>807</v>
       </c>
       <c r="D405" t="s">
-        <v>819</v>
+        <v>785</v>
       </c>
       <c r="E405" t="s">
-        <v>820</v>
+        <v>823</v>
       </c>
       <c r="F405" t="s">
-        <v>798</v>
+        <v>239</v>
       </c>
       <c r="G405" t="s">
-        <v>822</v>
+        <v>824</v>
       </c>
     </row>
     <row r="406" spans="1:7">
@@ -14377,16 +14377,16 @@
         <v>807</v>
       </c>
       <c r="D406" t="s">
-        <v>785</v>
+        <v>825</v>
       </c>
       <c r="E406" t="s">
-        <v>823</v>
+        <v>826</v>
       </c>
       <c r="F406" t="s">
-        <v>239</v>
+        <v>130</v>
       </c>
       <c r="G406" t="s">
-        <v>824</v>
+        <v>827</v>
       </c>
     </row>
     <row r="407" spans="1:7">
@@ -14400,16 +14400,16 @@
         <v>807</v>
       </c>
       <c r="D407" t="s">
-        <v>825</v>
+        <v>828</v>
       </c>
       <c r="E407" t="s">
-        <v>826</v>
+        <v>829</v>
       </c>
       <c r="F407" t="s">
         <v>130</v>
       </c>
       <c r="G407" t="s">
-        <v>827</v>
+        <v>830</v>
       </c>
     </row>
     <row r="408" spans="1:7">
@@ -14426,13 +14426,13 @@
         <v>828</v>
       </c>
       <c r="E408" t="s">
-        <v>829</v>
+        <v>831</v>
       </c>
       <c r="F408" t="s">
         <v>130</v>
       </c>
       <c r="G408" t="s">
-        <v>830</v>
+        <v>24</v>
       </c>
     </row>
     <row r="409" spans="1:7">
@@ -14443,19 +14443,19 @@
         <v>7</v>
       </c>
       <c r="C409" t="s">
-        <v>807</v>
+        <v>832</v>
       </c>
       <c r="D409" t="s">
-        <v>828</v>
+        <v>747</v>
       </c>
       <c r="E409" t="s">
-        <v>831</v>
+        <v>833</v>
       </c>
       <c r="F409" t="s">
-        <v>130</v>
+        <v>834</v>
       </c>
       <c r="G409" t="s">
-        <v>24</v>
+        <v>835</v>
       </c>
     </row>
     <row r="410" spans="1:7">
@@ -14475,10 +14475,10 @@
         <v>833</v>
       </c>
       <c r="F410" t="s">
-        <v>834</v>
+        <v>836</v>
       </c>
       <c r="G410" t="s">
-        <v>835</v>
+        <v>837</v>
       </c>
     </row>
     <row r="411" spans="1:7">
@@ -14495,13 +14495,13 @@
         <v>747</v>
       </c>
       <c r="E411" t="s">
-        <v>833</v>
+        <v>838</v>
       </c>
       <c r="F411" t="s">
-        <v>836</v>
+        <v>13</v>
       </c>
       <c r="G411" t="s">
-        <v>837</v>
+        <v>839</v>
       </c>
     </row>
     <row r="412" spans="1:7">
@@ -14515,16 +14515,16 @@
         <v>832</v>
       </c>
       <c r="D412" t="s">
-        <v>747</v>
+        <v>757</v>
       </c>
       <c r="E412" t="s">
-        <v>838</v>
+        <v>840</v>
       </c>
       <c r="F412" t="s">
-        <v>13</v>
+        <v>834</v>
       </c>
       <c r="G412" t="s">
-        <v>839</v>
+        <v>841</v>
       </c>
     </row>
     <row r="413" spans="1:7">
@@ -14544,10 +14544,10 @@
         <v>840</v>
       </c>
       <c r="F413" t="s">
-        <v>834</v>
+        <v>836</v>
       </c>
       <c r="G413" t="s">
-        <v>841</v>
+        <v>842</v>
       </c>
     </row>
     <row r="414" spans="1:7">
@@ -14567,10 +14567,10 @@
         <v>840</v>
       </c>
       <c r="F414" t="s">
-        <v>836</v>
+        <v>843</v>
       </c>
       <c r="G414" t="s">
-        <v>842</v>
+        <v>844</v>
       </c>
     </row>
     <row r="415" spans="1:7">
@@ -14590,10 +14590,10 @@
         <v>840</v>
       </c>
       <c r="F415" t="s">
-        <v>843</v>
+        <v>845</v>
       </c>
       <c r="G415" t="s">
-        <v>844</v>
+        <v>846</v>
       </c>
     </row>
     <row r="416" spans="1:7">
@@ -14607,16 +14607,16 @@
         <v>832</v>
       </c>
       <c r="D416" t="s">
-        <v>757</v>
+        <v>819</v>
       </c>
       <c r="E416" t="s">
-        <v>840</v>
+        <v>847</v>
       </c>
       <c r="F416" t="s">
-        <v>845</v>
+        <v>848</v>
       </c>
       <c r="G416" t="s">
-        <v>846</v>
+        <v>849</v>
       </c>
     </row>
     <row r="417" spans="1:7">
@@ -14630,16 +14630,16 @@
         <v>832</v>
       </c>
       <c r="D417" t="s">
-        <v>819</v>
+        <v>777</v>
       </c>
       <c r="E417" t="s">
-        <v>847</v>
+        <v>850</v>
       </c>
       <c r="F417" t="s">
-        <v>848</v>
+        <v>851</v>
       </c>
       <c r="G417" t="s">
-        <v>849</v>
+        <v>852</v>
       </c>
     </row>
     <row r="418" spans="1:7">
@@ -14653,16 +14653,16 @@
         <v>832</v>
       </c>
       <c r="D418" t="s">
-        <v>777</v>
+        <v>782</v>
       </c>
       <c r="E418" t="s">
-        <v>850</v>
+        <v>853</v>
       </c>
       <c r="F418" t="s">
-        <v>851</v>
+        <v>854</v>
       </c>
       <c r="G418" t="s">
-        <v>852</v>
+        <v>855</v>
       </c>
     </row>
     <row r="419" spans="1:7">
@@ -14676,16 +14676,16 @@
         <v>832</v>
       </c>
       <c r="D419" t="s">
-        <v>782</v>
+        <v>785</v>
       </c>
       <c r="E419" t="s">
-        <v>853</v>
+        <v>856</v>
       </c>
       <c r="F419" t="s">
         <v>854</v>
       </c>
       <c r="G419" t="s">
-        <v>855</v>
+        <v>857</v>
       </c>
     </row>
     <row r="420" spans="1:7">
@@ -14699,16 +14699,16 @@
         <v>832</v>
       </c>
       <c r="D420" t="s">
-        <v>785</v>
+        <v>800</v>
       </c>
       <c r="E420" t="s">
-        <v>856</v>
+        <v>858</v>
       </c>
       <c r="F420" t="s">
-        <v>854</v>
+        <v>627</v>
       </c>
       <c r="G420" t="s">
-        <v>857</v>
+        <v>859</v>
       </c>
     </row>
     <row r="421" spans="1:7">
@@ -14719,19 +14719,19 @@
         <v>7</v>
       </c>
       <c r="C421" t="s">
-        <v>832</v>
+        <v>860</v>
       </c>
       <c r="D421" t="s">
-        <v>800</v>
+        <v>747</v>
       </c>
       <c r="E421" t="s">
-        <v>858</v>
+        <v>861</v>
       </c>
       <c r="F421" t="s">
-        <v>627</v>
+        <v>834</v>
       </c>
       <c r="G421" t="s">
-        <v>859</v>
+        <v>862</v>
       </c>
     </row>
     <row r="422" spans="1:7">
@@ -14751,10 +14751,10 @@
         <v>861</v>
       </c>
       <c r="F422" t="s">
-        <v>834</v>
+        <v>836</v>
       </c>
       <c r="G422" t="s">
-        <v>862</v>
+        <v>863</v>
       </c>
     </row>
     <row r="423" spans="1:7">
@@ -14771,13 +14771,13 @@
         <v>747</v>
       </c>
       <c r="E423" t="s">
-        <v>861</v>
+        <v>864</v>
       </c>
       <c r="F423" t="s">
-        <v>836</v>
+        <v>15</v>
       </c>
       <c r="G423" t="s">
-        <v>863</v>
+        <v>865</v>
       </c>
     </row>
     <row r="424" spans="1:7">
@@ -14791,16 +14791,16 @@
         <v>860</v>
       </c>
       <c r="D424" t="s">
-        <v>747</v>
+        <v>866</v>
       </c>
       <c r="E424" t="s">
-        <v>864</v>
+        <v>867</v>
       </c>
       <c r="F424" t="s">
-        <v>15</v>
+        <v>834</v>
       </c>
       <c r="G424" t="s">
-        <v>865</v>
+        <v>868</v>
       </c>
     </row>
     <row r="425" spans="1:7">
@@ -14820,10 +14820,10 @@
         <v>867</v>
       </c>
       <c r="F425" t="s">
-        <v>834</v>
+        <v>836</v>
       </c>
       <c r="G425" t="s">
-        <v>868</v>
+        <v>869</v>
       </c>
     </row>
     <row r="426" spans="1:7">
@@ -14837,16 +14837,16 @@
         <v>860</v>
       </c>
       <c r="D426" t="s">
-        <v>866</v>
+        <v>757</v>
       </c>
       <c r="E426" t="s">
-        <v>867</v>
+        <v>870</v>
       </c>
       <c r="F426" t="s">
-        <v>836</v>
+        <v>854</v>
       </c>
       <c r="G426" t="s">
-        <v>869</v>
+        <v>871</v>
       </c>
     </row>
     <row r="427" spans="1:7">
@@ -14866,10 +14866,10 @@
         <v>870</v>
       </c>
       <c r="F427" t="s">
-        <v>854</v>
+        <v>845</v>
       </c>
       <c r="G427" t="s">
-        <v>871</v>
+        <v>872</v>
       </c>
     </row>
     <row r="428" spans="1:7">
@@ -14883,16 +14883,16 @@
         <v>860</v>
       </c>
       <c r="D428" t="s">
-        <v>757</v>
+        <v>762</v>
       </c>
       <c r="E428" t="s">
-        <v>870</v>
+        <v>873</v>
       </c>
       <c r="F428" t="s">
-        <v>845</v>
+        <v>874</v>
       </c>
       <c r="G428" t="s">
-        <v>872</v>
+        <v>875</v>
       </c>
     </row>
     <row r="429" spans="1:7">
@@ -14912,10 +14912,10 @@
         <v>873</v>
       </c>
       <c r="F429" t="s">
-        <v>874</v>
+        <v>854</v>
       </c>
       <c r="G429" t="s">
-        <v>875</v>
+        <v>876</v>
       </c>
     </row>
     <row r="430" spans="1:7">
@@ -14929,16 +14929,16 @@
         <v>860</v>
       </c>
       <c r="D430" t="s">
-        <v>762</v>
+        <v>819</v>
       </c>
       <c r="E430" t="s">
-        <v>873</v>
+        <v>877</v>
       </c>
       <c r="F430" t="s">
-        <v>854</v>
+        <v>836</v>
       </c>
       <c r="G430" t="s">
-        <v>876</v>
+        <v>878</v>
       </c>
     </row>
     <row r="431" spans="1:7">
@@ -14952,16 +14952,16 @@
         <v>860</v>
       </c>
       <c r="D431" t="s">
-        <v>819</v>
+        <v>828</v>
       </c>
       <c r="E431" t="s">
-        <v>877</v>
+        <v>879</v>
       </c>
       <c r="F431" t="s">
-        <v>836</v>
+        <v>15</v>
       </c>
       <c r="G431" t="s">
-        <v>878</v>
+        <v>880</v>
       </c>
     </row>
     <row r="432" spans="1:7">
@@ -14972,19 +14972,19 @@
         <v>7</v>
       </c>
       <c r="C432" t="s">
-        <v>860</v>
+        <v>881</v>
       </c>
       <c r="D432" t="s">
-        <v>828</v>
+        <v>747</v>
       </c>
       <c r="E432" t="s">
-        <v>879</v>
+        <v>882</v>
       </c>
       <c r="F432" t="s">
-        <v>15</v>
+        <v>883</v>
       </c>
       <c r="G432" t="s">
-        <v>880</v>
+        <v>872</v>
       </c>
     </row>
     <row r="433" spans="1:7">
@@ -15004,10 +15004,10 @@
         <v>882</v>
       </c>
       <c r="F433" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="G433" t="s">
-        <v>872</v>
+        <v>885</v>
       </c>
     </row>
     <row r="434" spans="1:7">
@@ -15027,10 +15027,10 @@
         <v>882</v>
       </c>
       <c r="F434" t="s">
-        <v>884</v>
+        <v>225</v>
       </c>
       <c r="G434" t="s">
-        <v>885</v>
+        <v>886</v>
       </c>
     </row>
     <row r="435" spans="1:7">
@@ -15050,10 +15050,10 @@
         <v>882</v>
       </c>
       <c r="F435" t="s">
-        <v>225</v>
+        <v>545</v>
       </c>
       <c r="G435" t="s">
-        <v>886</v>
+        <v>887</v>
       </c>
     </row>
     <row r="436" spans="1:7">
@@ -15067,16 +15067,16 @@
         <v>881</v>
       </c>
       <c r="D436" t="s">
-        <v>747</v>
+        <v>888</v>
       </c>
       <c r="E436" t="s">
-        <v>882</v>
+        <v>889</v>
       </c>
       <c r="F436" t="s">
-        <v>545</v>
+        <v>145</v>
       </c>
       <c r="G436" t="s">
-        <v>887</v>
+        <v>890</v>
       </c>
     </row>
     <row r="437" spans="1:7">
@@ -15093,13 +15093,13 @@
         <v>888</v>
       </c>
       <c r="E437" t="s">
-        <v>889</v>
+        <v>891</v>
       </c>
       <c r="F437" t="s">
         <v>145</v>
       </c>
       <c r="G437" t="s">
-        <v>890</v>
+        <v>892</v>
       </c>
     </row>
     <row r="438" spans="1:7">
@@ -15113,16 +15113,16 @@
         <v>881</v>
       </c>
       <c r="D438" t="s">
-        <v>888</v>
+        <v>893</v>
       </c>
       <c r="E438" t="s">
-        <v>891</v>
+        <v>894</v>
       </c>
       <c r="F438" t="s">
-        <v>145</v>
+        <v>895</v>
       </c>
       <c r="G438" t="s">
-        <v>892</v>
+        <v>896</v>
       </c>
     </row>
     <row r="439" spans="1:7">
@@ -15142,10 +15142,10 @@
         <v>894</v>
       </c>
       <c r="F439" t="s">
-        <v>895</v>
+        <v>225</v>
       </c>
       <c r="G439" t="s">
-        <v>896</v>
+        <v>897</v>
       </c>
     </row>
     <row r="440" spans="1:7">
@@ -15165,10 +15165,10 @@
         <v>894</v>
       </c>
       <c r="F440" t="s">
-        <v>225</v>
+        <v>898</v>
       </c>
       <c r="G440" t="s">
-        <v>897</v>
+        <v>899</v>
       </c>
     </row>
     <row r="441" spans="1:7">
@@ -15185,13 +15185,13 @@
         <v>893</v>
       </c>
       <c r="E441" t="s">
-        <v>894</v>
+        <v>900</v>
       </c>
       <c r="F441" t="s">
-        <v>898</v>
+        <v>545</v>
       </c>
       <c r="G441" t="s">
-        <v>899</v>
+        <v>901</v>
       </c>
     </row>
     <row r="442" spans="1:7">
@@ -15205,16 +15205,16 @@
         <v>881</v>
       </c>
       <c r="D442" t="s">
-        <v>893</v>
+        <v>902</v>
       </c>
       <c r="E442" t="s">
-        <v>900</v>
+        <v>903</v>
       </c>
       <c r="F442" t="s">
-        <v>545</v>
+        <v>883</v>
       </c>
       <c r="G442" t="s">
-        <v>901</v>
+        <v>904</v>
       </c>
     </row>
     <row r="443" spans="1:7">
@@ -15234,10 +15234,10 @@
         <v>903</v>
       </c>
       <c r="F443" t="s">
-        <v>883</v>
+        <v>225</v>
       </c>
       <c r="G443" t="s">
-        <v>904</v>
+        <v>905</v>
       </c>
     </row>
     <row r="444" spans="1:7">
@@ -15257,10 +15257,10 @@
         <v>903</v>
       </c>
       <c r="F444" t="s">
-        <v>225</v>
+        <v>545</v>
       </c>
       <c r="G444" t="s">
-        <v>905</v>
+        <v>906</v>
       </c>
     </row>
     <row r="445" spans="1:7">
@@ -15277,13 +15277,13 @@
         <v>902</v>
       </c>
       <c r="E445" t="s">
-        <v>903</v>
+        <v>907</v>
       </c>
       <c r="F445" t="s">
-        <v>545</v>
+        <v>883</v>
       </c>
       <c r="G445" t="s">
-        <v>906</v>
+        <v>908</v>
       </c>
     </row>
     <row r="446" spans="1:7">
@@ -15303,10 +15303,10 @@
         <v>907</v>
       </c>
       <c r="F446" t="s">
-        <v>883</v>
+        <v>225</v>
       </c>
       <c r="G446" t="s">
-        <v>908</v>
+        <v>909</v>
       </c>
     </row>
     <row r="447" spans="1:7">
@@ -15326,10 +15326,10 @@
         <v>907</v>
       </c>
       <c r="F447" t="s">
-        <v>225</v>
+        <v>568</v>
       </c>
       <c r="G447" t="s">
-        <v>909</v>
+        <v>910</v>
       </c>
     </row>
     <row r="448" spans="1:7">
@@ -15343,16 +15343,16 @@
         <v>881</v>
       </c>
       <c r="D448" t="s">
-        <v>902</v>
+        <v>782</v>
       </c>
       <c r="E448" t="s">
-        <v>907</v>
+        <v>911</v>
       </c>
       <c r="F448" t="s">
-        <v>568</v>
+        <v>545</v>
       </c>
       <c r="G448" t="s">
-        <v>910</v>
+        <v>912</v>
       </c>
     </row>
     <row r="449" spans="1:7">
@@ -15366,16 +15366,16 @@
         <v>881</v>
       </c>
       <c r="D449" t="s">
-        <v>782</v>
+        <v>785</v>
       </c>
       <c r="E449" t="s">
-        <v>911</v>
+        <v>913</v>
       </c>
       <c r="F449" t="s">
-        <v>545</v>
+        <v>225</v>
       </c>
       <c r="G449" t="s">
-        <v>912</v>
+        <v>914</v>
       </c>
     </row>
     <row r="450" spans="1:7">
@@ -15389,16 +15389,16 @@
         <v>881</v>
       </c>
       <c r="D450" t="s">
-        <v>785</v>
+        <v>915</v>
       </c>
       <c r="E450" t="s">
-        <v>913</v>
+        <v>916</v>
       </c>
       <c r="F450" t="s">
-        <v>225</v>
+        <v>145</v>
       </c>
       <c r="G450" t="s">
-        <v>914</v>
+        <v>917</v>
       </c>
     </row>
     <row r="451" spans="1:7">
@@ -15412,16 +15412,16 @@
         <v>881</v>
       </c>
       <c r="D451" t="s">
-        <v>915</v>
+        <v>918</v>
       </c>
       <c r="E451" t="s">
-        <v>916</v>
+        <v>919</v>
       </c>
       <c r="F451" t="s">
-        <v>145</v>
+        <v>809</v>
       </c>
       <c r="G451" t="s">
-        <v>917</v>
+        <v>920</v>
       </c>
     </row>
     <row r="452" spans="1:7">
@@ -15432,19 +15432,19 @@
         <v>7</v>
       </c>
       <c r="C452" t="s">
-        <v>881</v>
+        <v>921</v>
       </c>
       <c r="D452" t="s">
-        <v>918</v>
+        <v>922</v>
       </c>
       <c r="E452" t="s">
-        <v>919</v>
+        <v>923</v>
       </c>
       <c r="F452" t="s">
-        <v>809</v>
+        <v>174</v>
       </c>
       <c r="G452" t="s">
-        <v>920</v>
+        <v>924</v>
       </c>
     </row>
     <row r="453" spans="1:7">
@@ -15458,16 +15458,16 @@
         <v>921</v>
       </c>
       <c r="D453" t="s">
-        <v>922</v>
+        <v>925</v>
       </c>
       <c r="E453" t="s">
-        <v>923</v>
+        <v>926</v>
       </c>
       <c r="F453" t="s">
         <v>174</v>
       </c>
       <c r="G453" t="s">
-        <v>924</v>
+        <v>927</v>
       </c>
     </row>
     <row r="454" spans="1:7">
@@ -15487,10 +15487,10 @@
         <v>926</v>
       </c>
       <c r="F454" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="G454" t="s">
-        <v>927</v>
+        <v>928</v>
       </c>
     </row>
     <row r="455" spans="1:7">
@@ -15507,13 +15507,13 @@
         <v>925</v>
       </c>
       <c r="E455" t="s">
-        <v>926</v>
+        <v>929</v>
       </c>
       <c r="F455" t="s">
-        <v>163</v>
+        <v>174</v>
       </c>
       <c r="G455" t="s">
-        <v>928</v>
+        <v>930</v>
       </c>
     </row>
     <row r="456" spans="1:7">
@@ -15533,10 +15533,10 @@
         <v>929</v>
       </c>
       <c r="F456" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="G456" t="s">
-        <v>930</v>
+        <v>931</v>
       </c>
     </row>
     <row r="457" spans="1:7">
@@ -15553,13 +15553,13 @@
         <v>925</v>
       </c>
       <c r="E457" t="s">
-        <v>929</v>
+        <v>932</v>
       </c>
       <c r="F457" t="s">
-        <v>163</v>
+        <v>933</v>
       </c>
       <c r="G457" t="s">
-        <v>931</v>
+        <v>934</v>
       </c>
     </row>
     <row r="458" spans="1:7">
@@ -15576,13 +15576,13 @@
         <v>925</v>
       </c>
       <c r="E458" t="s">
-        <v>932</v>
+        <v>935</v>
       </c>
       <c r="F458" t="s">
-        <v>933</v>
+        <v>174</v>
       </c>
       <c r="G458" t="s">
-        <v>934</v>
+        <v>936</v>
       </c>
     </row>
     <row r="459" spans="1:7">
@@ -15602,10 +15602,10 @@
         <v>935</v>
       </c>
       <c r="F459" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="G459" t="s">
-        <v>936</v>
+        <v>937</v>
       </c>
     </row>
     <row r="460" spans="1:7">
@@ -15622,13 +15622,13 @@
         <v>925</v>
       </c>
       <c r="E460" t="s">
-        <v>935</v>
+        <v>938</v>
       </c>
       <c r="F460" t="s">
-        <v>163</v>
+        <v>174</v>
       </c>
       <c r="G460" t="s">
-        <v>937</v>
+        <v>939</v>
       </c>
     </row>
     <row r="461" spans="1:7">
@@ -15648,10 +15648,10 @@
         <v>938</v>
       </c>
       <c r="F461" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="G461" t="s">
-        <v>939</v>
+        <v>940</v>
       </c>
     </row>
     <row r="462" spans="1:7">
@@ -15668,13 +15668,13 @@
         <v>925</v>
       </c>
       <c r="E462" t="s">
-        <v>938</v>
+        <v>941</v>
       </c>
       <c r="F462" t="s">
-        <v>163</v>
+        <v>933</v>
       </c>
       <c r="G462" t="s">
-        <v>940</v>
+        <v>942</v>
       </c>
     </row>
     <row r="463" spans="1:7">
@@ -15688,16 +15688,16 @@
         <v>921</v>
       </c>
       <c r="D463" t="s">
-        <v>925</v>
+        <v>943</v>
       </c>
       <c r="E463" t="s">
-        <v>941</v>
+        <v>944</v>
       </c>
       <c r="F463" t="s">
-        <v>933</v>
+        <v>174</v>
       </c>
       <c r="G463" t="s">
-        <v>942</v>
+        <v>945</v>
       </c>
     </row>
     <row r="464" spans="1:7">
@@ -15717,10 +15717,10 @@
         <v>944</v>
       </c>
       <c r="F464" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="G464" t="s">
-        <v>945</v>
+        <v>946</v>
       </c>
     </row>
     <row r="465" spans="1:7">
@@ -15734,16 +15734,16 @@
         <v>921</v>
       </c>
       <c r="D465" t="s">
-        <v>943</v>
+        <v>947</v>
       </c>
       <c r="E465" t="s">
-        <v>944</v>
+        <v>948</v>
       </c>
       <c r="F465" t="s">
-        <v>163</v>
+        <v>503</v>
       </c>
       <c r="G465" t="s">
-        <v>946</v>
+        <v>949</v>
       </c>
     </row>
     <row r="466" spans="1:7">
@@ -15763,10 +15763,10 @@
         <v>948</v>
       </c>
       <c r="F466" t="s">
-        <v>503</v>
+        <v>933</v>
       </c>
       <c r="G466" t="s">
-        <v>949</v>
+        <v>950</v>
       </c>
     </row>
     <row r="467" spans="1:7">
@@ -15786,10 +15786,10 @@
         <v>948</v>
       </c>
       <c r="F467" t="s">
-        <v>933</v>
+        <v>174</v>
       </c>
       <c r="G467" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
     </row>
     <row r="468" spans="1:7">
@@ -15809,10 +15809,10 @@
         <v>948</v>
       </c>
       <c r="F468" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="G468" t="s">
-        <v>951</v>
+        <v>466</v>
       </c>
     </row>
     <row r="469" spans="1:7">
@@ -15826,16 +15826,16 @@
         <v>921</v>
       </c>
       <c r="D469" t="s">
-        <v>947</v>
+        <v>952</v>
       </c>
       <c r="E469" t="s">
-        <v>948</v>
+        <v>953</v>
       </c>
       <c r="F469" t="s">
-        <v>163</v>
+        <v>933</v>
       </c>
       <c r="G469" t="s">
-        <v>466</v>
+        <v>45</v>
       </c>
     </row>
     <row r="470" spans="1:7">
@@ -15855,10 +15855,10 @@
         <v>953</v>
       </c>
       <c r="F470" t="s">
-        <v>933</v>
+        <v>163</v>
       </c>
       <c r="G470" t="s">
-        <v>45</v>
+        <v>954</v>
       </c>
     </row>
     <row r="471" spans="1:7">
@@ -15872,16 +15872,16 @@
         <v>921</v>
       </c>
       <c r="D471" t="s">
-        <v>952</v>
+        <v>955</v>
       </c>
       <c r="E471" t="s">
-        <v>953</v>
+        <v>956</v>
       </c>
       <c r="F471" t="s">
-        <v>163</v>
+        <v>883</v>
       </c>
       <c r="G471" t="s">
-        <v>954</v>
+        <v>957</v>
       </c>
     </row>
     <row r="472" spans="1:7">
@@ -15901,10 +15901,10 @@
         <v>956</v>
       </c>
       <c r="F472" t="s">
-        <v>883</v>
+        <v>933</v>
       </c>
       <c r="G472" t="s">
-        <v>957</v>
+        <v>958</v>
       </c>
     </row>
     <row r="473" spans="1:7">
@@ -15924,10 +15924,10 @@
         <v>956</v>
       </c>
       <c r="F473" t="s">
-        <v>933</v>
+        <v>174</v>
       </c>
       <c r="G473" t="s">
-        <v>958</v>
+        <v>45</v>
       </c>
     </row>
     <row r="474" spans="1:7">
@@ -15947,10 +15947,10 @@
         <v>956</v>
       </c>
       <c r="F474" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="G474" t="s">
-        <v>45</v>
+        <v>959</v>
       </c>
     </row>
     <row r="475" spans="1:7">
@@ -15964,16 +15964,16 @@
         <v>921</v>
       </c>
       <c r="D475" t="s">
-        <v>955</v>
+        <v>960</v>
       </c>
       <c r="E475" t="s">
-        <v>956</v>
+        <v>961</v>
       </c>
       <c r="F475" t="s">
-        <v>163</v>
+        <v>933</v>
       </c>
       <c r="G475" t="s">
-        <v>959</v>
+        <v>45</v>
       </c>
     </row>
     <row r="476" spans="1:7">
@@ -15993,10 +15993,10 @@
         <v>961</v>
       </c>
       <c r="F476" t="s">
-        <v>933</v>
+        <v>174</v>
       </c>
       <c r="G476" t="s">
-        <v>45</v>
+        <v>962</v>
       </c>
     </row>
     <row r="477" spans="1:7">
@@ -16010,16 +16010,16 @@
         <v>921</v>
       </c>
       <c r="D477" t="s">
-        <v>960</v>
+        <v>963</v>
       </c>
       <c r="E477" t="s">
-        <v>961</v>
+        <v>964</v>
       </c>
       <c r="F477" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="G477" t="s">
-        <v>962</v>
+        <v>965</v>
       </c>
     </row>
     <row r="478" spans="1:7">
@@ -16033,16 +16033,16 @@
         <v>921</v>
       </c>
       <c r="D478" t="s">
-        <v>963</v>
+        <v>966</v>
       </c>
       <c r="E478" t="s">
-        <v>964</v>
+        <v>967</v>
       </c>
       <c r="F478" t="s">
-        <v>163</v>
+        <v>174</v>
       </c>
       <c r="G478" t="s">
-        <v>965</v>
+        <v>968</v>
       </c>
     </row>
     <row r="479" spans="1:7">
@@ -16062,10 +16062,10 @@
         <v>967</v>
       </c>
       <c r="F479" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="G479" t="s">
-        <v>968</v>
+        <v>969</v>
       </c>
     </row>
     <row r="480" spans="1:7">
@@ -16079,16 +16079,16 @@
         <v>921</v>
       </c>
       <c r="D480" t="s">
-        <v>966</v>
+        <v>43</v>
       </c>
       <c r="E480" t="s">
-        <v>967</v>
+        <v>970</v>
       </c>
       <c r="F480" t="s">
-        <v>163</v>
+        <v>933</v>
       </c>
       <c r="G480" t="s">
-        <v>969</v>
+        <v>45</v>
       </c>
     </row>
     <row r="481" spans="1:7">
@@ -16108,10 +16108,10 @@
         <v>970</v>
       </c>
       <c r="F481" t="s">
-        <v>933</v>
+        <v>163</v>
       </c>
       <c r="G481" t="s">
-        <v>45</v>
+        <v>127</v>
       </c>
     </row>
     <row r="482" spans="1:7">
@@ -16125,16 +16125,16 @@
         <v>921</v>
       </c>
       <c r="D482" t="s">
-        <v>43</v>
+        <v>971</v>
       </c>
       <c r="E482" t="s">
-        <v>970</v>
+        <v>972</v>
       </c>
       <c r="F482" t="s">
-        <v>163</v>
+        <v>933</v>
       </c>
       <c r="G482" t="s">
-        <v>127</v>
+        <v>45</v>
       </c>
     </row>
     <row r="483" spans="1:7">
@@ -16154,7 +16154,7 @@
         <v>972</v>
       </c>
       <c r="F483" t="s">
-        <v>933</v>
+        <v>174</v>
       </c>
       <c r="G483" t="s">
         <v>45</v>
@@ -16171,16 +16171,16 @@
         <v>921</v>
       </c>
       <c r="D484" t="s">
-        <v>971</v>
+        <v>973</v>
       </c>
       <c r="E484" t="s">
-        <v>972</v>
+        <v>974</v>
       </c>
       <c r="F484" t="s">
-        <v>174</v>
+        <v>933</v>
       </c>
       <c r="G484" t="s">
-        <v>45</v>
+        <v>975</v>
       </c>
     </row>
     <row r="485" spans="1:7">
@@ -16191,19 +16191,19 @@
         <v>7</v>
       </c>
       <c r="C485" t="s">
-        <v>921</v>
+        <v>976</v>
       </c>
       <c r="D485" t="s">
-        <v>973</v>
+        <v>925</v>
       </c>
       <c r="E485" t="s">
-        <v>974</v>
+        <v>977</v>
       </c>
       <c r="F485" t="s">
-        <v>933</v>
+        <v>174</v>
       </c>
       <c r="G485" t="s">
-        <v>975</v>
+        <v>978</v>
       </c>
     </row>
     <row r="486" spans="1:7">
@@ -16223,10 +16223,10 @@
         <v>977</v>
       </c>
       <c r="F486" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="G486" t="s">
-        <v>978</v>
+        <v>979</v>
       </c>
     </row>
     <row r="487" spans="1:7">
@@ -16243,13 +16243,13 @@
         <v>925</v>
       </c>
       <c r="E487" t="s">
-        <v>977</v>
+        <v>980</v>
       </c>
       <c r="F487" t="s">
-        <v>163</v>
+        <v>174</v>
       </c>
       <c r="G487" t="s">
-        <v>979</v>
+        <v>981</v>
       </c>
     </row>
     <row r="488" spans="1:7">
@@ -16269,10 +16269,10 @@
         <v>980</v>
       </c>
       <c r="F488" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="G488" t="s">
-        <v>981</v>
+        <v>982</v>
       </c>
     </row>
     <row r="489" spans="1:7">
@@ -16289,13 +16289,13 @@
         <v>925</v>
       </c>
       <c r="E489" t="s">
-        <v>980</v>
+        <v>983</v>
       </c>
       <c r="F489" t="s">
-        <v>163</v>
+        <v>933</v>
       </c>
       <c r="G489" t="s">
-        <v>982</v>
+        <v>959</v>
       </c>
     </row>
     <row r="490" spans="1:7">
@@ -16309,16 +16309,16 @@
         <v>976</v>
       </c>
       <c r="D490" t="s">
-        <v>925</v>
+        <v>947</v>
       </c>
       <c r="E490" t="s">
-        <v>983</v>
+        <v>984</v>
       </c>
       <c r="F490" t="s">
         <v>933</v>
       </c>
       <c r="G490" t="s">
-        <v>959</v>
+        <v>985</v>
       </c>
     </row>
     <row r="491" spans="1:7">
@@ -16338,10 +16338,10 @@
         <v>984</v>
       </c>
       <c r="F491" t="s">
-        <v>933</v>
+        <v>174</v>
       </c>
       <c r="G491" t="s">
-        <v>985</v>
+        <v>986</v>
       </c>
     </row>
     <row r="492" spans="1:7">
@@ -16361,10 +16361,10 @@
         <v>984</v>
       </c>
       <c r="F492" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="G492" t="s">
-        <v>986</v>
+        <v>987</v>
       </c>
     </row>
     <row r="493" spans="1:7">
@@ -16378,16 +16378,16 @@
         <v>976</v>
       </c>
       <c r="D493" t="s">
-        <v>947</v>
+        <v>955</v>
       </c>
       <c r="E493" t="s">
-        <v>984</v>
+        <v>988</v>
       </c>
       <c r="F493" t="s">
-        <v>163</v>
+        <v>933</v>
       </c>
       <c r="G493" t="s">
-        <v>987</v>
+        <v>989</v>
       </c>
     </row>
     <row r="494" spans="1:7">
@@ -16407,10 +16407,10 @@
         <v>988</v>
       </c>
       <c r="F494" t="s">
-        <v>933</v>
+        <v>174</v>
       </c>
       <c r="G494" t="s">
-        <v>989</v>
+        <v>45</v>
       </c>
     </row>
     <row r="495" spans="1:7">
@@ -16430,10 +16430,10 @@
         <v>988</v>
       </c>
       <c r="F495" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="G495" t="s">
-        <v>45</v>
+        <v>942</v>
       </c>
     </row>
     <row r="496" spans="1:7">
@@ -16447,16 +16447,16 @@
         <v>976</v>
       </c>
       <c r="D496" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="E496" t="s">
-        <v>988</v>
+        <v>990</v>
       </c>
       <c r="F496" t="s">
-        <v>163</v>
+        <v>933</v>
       </c>
       <c r="G496" t="s">
-        <v>942</v>
+        <v>991</v>
       </c>
     </row>
     <row r="497" spans="1:7">
@@ -16476,10 +16476,10 @@
         <v>990</v>
       </c>
       <c r="F497" t="s">
-        <v>933</v>
+        <v>163</v>
       </c>
       <c r="G497" t="s">
-        <v>991</v>
+        <v>992</v>
       </c>
     </row>
     <row r="498" spans="1:7">
@@ -16493,16 +16493,16 @@
         <v>976</v>
       </c>
       <c r="D498" t="s">
-        <v>963</v>
+        <v>43</v>
       </c>
       <c r="E498" t="s">
-        <v>990</v>
+        <v>993</v>
       </c>
       <c r="F498" t="s">
-        <v>163</v>
+        <v>933</v>
       </c>
       <c r="G498" t="s">
-        <v>992</v>
+        <v>45</v>
       </c>
     </row>
     <row r="499" spans="1:7">
@@ -16522,7 +16522,7 @@
         <v>993</v>
       </c>
       <c r="F499" t="s">
-        <v>933</v>
+        <v>163</v>
       </c>
       <c r="G499" t="s">
         <v>45</v>
@@ -16539,38 +16539,15 @@
         <v>976</v>
       </c>
       <c r="D500" t="s">
-        <v>43</v>
+        <v>971</v>
       </c>
       <c r="E500" t="s">
-        <v>993</v>
+        <v>972</v>
       </c>
       <c r="F500" t="s">
         <v>163</v>
       </c>
       <c r="G500" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="501" spans="1:7">
-      <c r="A501">
-        <v>500</v>
-      </c>
-      <c r="B501" t="s">
-        <v>7</v>
-      </c>
-      <c r="C501" t="s">
-        <v>976</v>
-      </c>
-      <c r="D501" t="s">
-        <v>971</v>
-      </c>
-      <c r="E501" t="s">
-        <v>972</v>
-      </c>
-      <c r="F501" t="s">
-        <v>163</v>
-      </c>
-      <c r="G501" t="s">
         <v>45</v>
       </c>
     </row>

</xml_diff>